<commit_message>
update[research]: Adding new papers in the list of research papers excel sheet.
</commit_message>
<xml_diff>
--- a/research/List of Research Papers.xlsx
+++ b/research/List of Research Papers.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gamin\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B31A9DC2-5D0B-4D3C-87EF-557B6401A626}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{343B6B6F-B0CA-4653-B191-2D86EBBA5ED1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{01C390C4-20FF-4F65-BB66-A7A558CEAB89}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="63">
   <si>
     <t>Sl. No.</t>
   </si>
@@ -171,6 +171,60 @@
   </si>
   <si>
     <t>Deep learning-based flood detection system using semantic segmentation</t>
+  </si>
+  <si>
+    <t>Flood prediction using Time Series Data Mining</t>
+  </si>
+  <si>
+    <t>https://www.sciencedirect.com/science/article/abs/pii/S0022169406004331</t>
+  </si>
+  <si>
+    <t>flood prediction using time series</t>
+  </si>
+  <si>
+    <t>https://www.mdpi.com/2073-4441/12/1/96</t>
+  </si>
+  <si>
+    <t>Convolutional neural network coupled with a transfer-learning approach for time-series flood predictions</t>
+  </si>
+  <si>
+    <t>https://www.sciencedirect.com/science/article/pii/S0022169423006443</t>
+  </si>
+  <si>
+    <t>Time-series generative adversarial networks for flood forecasting</t>
+  </si>
+  <si>
+    <t>Context-based Hydrology Time Series Data for A Flood Prediction Model Using LSTM</t>
+  </si>
+  <si>
+    <t>https://ieeexplore.ieee.org/document/8576900/</t>
+  </si>
+  <si>
+    <t>Deep Learning Based Spatio-Temporal Modeling for Flood Risk Prediction in Jakarta</t>
+  </si>
+  <si>
+    <t>https://ieeexplore.ieee.org/document/11393369/</t>
+  </si>
+  <si>
+    <t>hybrid neural network architectures for flood prediction</t>
+  </si>
+  <si>
+    <t>Flood Prediction Using LSTM with Other Deep Learning Architecture</t>
+  </si>
+  <si>
+    <t>https://ieeexplore.ieee.org/document/10918361/</t>
+  </si>
+  <si>
+    <t>Early classification of industrial alarm floods using a hybrid neural network and optimal time-encoded histograms</t>
+  </si>
+  <si>
+    <t>https://www.sciencedirect.com/science/article/abs/pii/S0952197625037376</t>
+  </si>
+  <si>
+    <t>A Hybrid Deep Learning Approach Using Vision Transformer and U-Net for Flood Segmentation</t>
+  </si>
+  <si>
+    <t>https://www.sciencedirect.com/science/article/pii/S1546221825012512</t>
   </si>
 </sst>
 </file>
@@ -556,7 +610,7 @@
   <cols>
     <col min="2" max="2" width="98.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="255.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="47" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -832,77 +886,173 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B17" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" t="s">
+        <v>47</v>
+      </c>
+      <c r="E17" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B18" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" t="s">
+        <v>48</v>
+      </c>
+      <c r="D18" t="s">
+        <v>47</v>
+      </c>
+      <c r="E18" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B19" t="s">
+        <v>51</v>
+      </c>
+      <c r="C19" t="s">
+        <v>50</v>
+      </c>
+      <c r="D19" t="s">
+        <v>47</v>
+      </c>
+      <c r="E19" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B20" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" t="s">
+        <v>53</v>
+      </c>
+      <c r="D20" t="s">
+        <v>47</v>
+      </c>
+      <c r="E20" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B21" t="s">
+        <v>54</v>
+      </c>
+      <c r="C21" t="s">
+        <v>55</v>
+      </c>
+      <c r="D21" t="s">
+        <v>56</v>
+      </c>
+      <c r="E21" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B22" t="s">
+        <v>57</v>
+      </c>
+      <c r="C22" t="s">
+        <v>58</v>
+      </c>
+      <c r="D22" t="s">
+        <v>56</v>
+      </c>
+      <c r="E22" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C23" t="s">
+        <v>60</v>
+      </c>
+      <c r="D23" t="s">
+        <v>56</v>
+      </c>
+      <c r="E23" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B24" t="s">
+        <v>61</v>
+      </c>
+      <c r="C24" t="s">
+        <v>62</v>
+      </c>
+      <c r="D24" t="s">
+        <v>56</v>
+      </c>
+      <c r="E24" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>

</xml_diff>

<commit_message>
update[research]: Adding some research papers to the list for the reference. - Daiwik
</commit_message>
<xml_diff>
--- a/research/List of Research Papers.xlsx
+++ b/research/List of Research Papers.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gamin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Daiwik VIT\EPICS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{343B6B6F-B0CA-4653-B191-2D86EBBA5ED1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{218C1830-A016-4DE0-98CF-2E5CAAB1BDD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{01C390C4-20FF-4F65-BB66-A7A558CEAB89}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{01C390C4-20FF-4F65-BB66-A7A558CEAB89}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="84">
   <si>
     <t>Sl. No.</t>
   </si>
@@ -225,13 +223,76 @@
   </si>
   <si>
     <t>https://www.sciencedirect.com/science/article/pii/S1546221825012512</t>
+  </si>
+  <si>
+    <t>A novel framework embedding Bayesian-optimized ensemble machine learning and explainable artificial intelligence (XAI) to improve flood prediction in complex watersheds</t>
+  </si>
+  <si>
+    <t>https://www.sciencedirect.com/science/article/pii/S2665972725001813</t>
+  </si>
+  <si>
+    <t>flood prediction ensemble machine learning SHAP watershed</t>
+  </si>
+  <si>
+    <t>Deep learning of flood forecasting by considering interpretability and physical constraints</t>
+  </si>
+  <si>
+    <t>https://hess.copernicus.org/articles/29/5955/2025/</t>
+  </si>
+  <si>
+    <t>interpretable deep learning flood forecasting physical constraints</t>
+  </si>
+  <si>
+    <t>Predicting Flood Potential Using Machine Learning with the XGBoost and Logistic Regression Approaches</t>
+  </si>
+  <si>
+    <t>https://jurnal.umb.ac.id/index.php/JSAI/article/view/9867</t>
+  </si>
+  <si>
+    <t>XGBoost flood prediction weather data classification</t>
+  </si>
+  <si>
+    <t>Machine Learning Models for Predicting Flood Events Using Weather Data: An Evaluation of Logistic Regression, LightGBM, and XGBoost</t>
+  </si>
+  <si>
+    <t>https://www.bright-journal.org/Journal/index.php/JADS/article/view/503</t>
+  </si>
+  <si>
+    <t>LightGBM flood prediction comparison XGBoost accuracy</t>
+  </si>
+  <si>
+    <t>Predicting peak inundation depths with a physics informed machine learning model</t>
+  </si>
+  <si>
+    <t>Combining Machine Learning Models and Satellite Data of an Extreme Flood Event for Flood Susceptibility Mapping</t>
+  </si>
+  <si>
+    <t>Beyond Observed Extremes: Can Hybrid Deep Learning Models Improve Flood Prediction?</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/s41598-024-65570-8</t>
+  </si>
+  <si>
+    <t>https://www.mdpi.com/2073-4441/17/18/2678</t>
+  </si>
+  <si>
+    <t>https://egusphere.copernicus.org/preprints/2025/egusphere-2025-1509/</t>
+  </si>
+  <si>
+    <t>physics informed machine learning flood depth prediction</t>
+  </si>
+  <si>
+    <t>satellite data flood susceptibility random forest XGBoost</t>
+  </si>
+  <si>
+    <t>hybrid deep learning flood prediction LSTM hydrology</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -243,6 +304,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -265,14 +334,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1026,38 +1098,125 @@
       <c r="A25">
         <v>24</v>
       </c>
+      <c r="B25" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" t="s">
+        <v>64</v>
+      </c>
+      <c r="D25" t="s">
+        <v>65</v>
+      </c>
+      <c r="E25" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
+      <c r="B26" t="s">
+        <v>66</v>
+      </c>
+      <c r="C26" t="s">
+        <v>67</v>
+      </c>
+      <c r="D26" t="s">
+        <v>68</v>
+      </c>
+      <c r="E26" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
+      <c r="B27" t="s">
+        <v>69</v>
+      </c>
+      <c r="C27" t="s">
+        <v>70</v>
+      </c>
+      <c r="D27" t="s">
+        <v>71</v>
+      </c>
+      <c r="E27" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
+      <c r="B28" t="s">
+        <v>72</v>
+      </c>
+      <c r="C28" t="s">
+        <v>73</v>
+      </c>
+      <c r="D28" t="s">
+        <v>74</v>
+      </c>
+      <c r="E28" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
+      <c r="B29" t="s">
+        <v>75</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D29" t="s">
+        <v>81</v>
+      </c>
+      <c r="E29" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
+      <c r="B30" t="s">
+        <v>76</v>
+      </c>
+      <c r="C30" t="s">
+        <v>79</v>
+      </c>
+      <c r="D30" t="s">
+        <v>82</v>
+      </c>
+      <c r="E30" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
+      <c r="B31" t="s">
+        <v>77</v>
+      </c>
+      <c r="C31" t="s">
+        <v>80</v>
+      </c>
+      <c r="D31" t="s">
+        <v>83</v>
+      </c>
+      <c r="E31" t="s">
+        <v>30</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C29" r:id="rId1" xr:uid="{BF63AC7D-2EFE-487F-A938-BD3E06AF6E88}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>